<commit_message>
Add eleven reviewed SCUT academic profiles with school-chunk conservation
</commit_message>
<xml_diff>
--- a/site/exports/scut-math.xlsx
+++ b/site/exports/scut-math.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -675,12 +675,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>钟友良</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>数学学院</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>https://www2.scut.edu.cn/math/2018/0316/c14638a440128/page.htm</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>仅依据已留存的必要职业摘录，非完整网页或完整履历；未独立核实当前人事状态，任职导航关闭。；原学位证书、学位论文与论文全文未读取；不由学习结束年月推断授位日期。；官方数学学院简介置副教授栏目；该标签未给任期，2017至2019年是数学学院博士后期间，不是副教授任期。；原页发布时间2018-03-16，正文有2019年区间结束；发布时间不等内容最后更新日期。；招生专业：基础数学；不据此添加未明示的硕导或博导资格。；研究方向：曲面的Teichmüller空间与模空间的度量结构；原文链接至MathSciNet的工作未跟随，未留存具体作品题名。；本科与硕博均保留学习阶段；硕博不拆两个授位；本人导师与完整作品未知。；数学学院展示复用本校既有单位；本次个人页不是独立目录或实时人事核验。</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K4"/>
+  <autoFilter ref="A1:K5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -692,11 +746,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="32.2" customWidth="1" min="2" max="2"/>
+    <col width="40.59999999999999" customWidth="1" min="2" max="2"/>
     <col width="23.8" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -2241,8 +2295,333 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>钟友良</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>education_label_award_unknown</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>中山大学</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>信息与计算科学</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>保留来源学习阶段与学位称谓；授位状态及证书未单独核实。 学习区间不当授位日期。 来源单位标签：数学与计算科学。该院系标签不替代本人专业或独立授位机构认定。</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://www2.scut.edu.cn/math/2018/0316/c14638a440128/page.htm</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>钟友良</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>education_label_award_unknown</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>硕博</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>中山大学</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>基础数学</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>来源仅列硕博合并学习阶段，不拆成两项授位；具体授位及授位时间未核。 来源单位标签：数学与计算科学。该院系标签不替代本人专业或独立授位机构认定。</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://www2.scut.edu.cn/math/2018/0316/c14638a440128/page.htm</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>钟友良</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_training</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>博士后</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>复旦大学</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>来源列示博士后研究，非学位事件；研究机构和区间按原文保留。 来源单位标签：上海数学中心。该院系标签不替代本人专业或独立授位机构认定。</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://www2.scut.edu.cn/math/2018/0316/c14638a440128/page.htm</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>钟友良</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>nondegree_training</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>博士后</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>来源列示博士后研究，非学位事件；研究机构和区间按原文保留。 来源单位标签：数学学院。该院系标签不替代本人专业或独立授位机构认定。</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://www2.scut.edu.cn/math/2018/0316/c14638a440128/page.htm</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>钟友良</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>副教授（页面栏目）</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学数学学院</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>来源副教授栏目标签；未给任期，不将历史博士后区间当副教授任期。</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://www2.scut.edu.cn/math/2018/0316/c14638a440128/page.htm</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S21"/>
+  <autoFilter ref="A1:S26"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -2264,6 +2643,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3132,7 +3516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3591,27 +3975,23 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>陈博聪</t>
+          <t>钟友良</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>institution-classification-4</t>
+          <t>scut-zhong-388</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
-        </is>
-      </c>
+          <t>https://www2.scut.edu.cn/math/2018/0316/c14638a440128/page.htm</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>未单独记录</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -3628,17 +4008,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>陈培</t>
+          <t>陈博聪</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>institution-classification-2</t>
+          <t>institution-classification-4</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>https://xxgk.scut.edu.cn/_upload/article/files/f9/59/7229d8c64109b93efc60864c9f8f/715ab56f-79b5-46ff-afae-c75af81b2036.pdf</t>
+          <t>https://www.moe.gov.cn/srcsite/A22/s7065/200612/t20061206_128833.html</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -3665,42 +4045,79 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>陈培</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>institution-classification-2</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>https://xxgk.scut.edu.cn/_upload/article/files/f9/59/7229d8c64109b93efc60864c9f8f/715ab56f-79b5-46ff-afae-c75af81b2036.pdf</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>未单独记录</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>华南理工大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>陈映珊</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>institution-classification-5</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>https://xxgk.scut.edu.cn/_upload/article/files/f9/59/7229d8c64109b93efc60864c9f8f/715ab56f-79b5-46ff-afae-c75af81b2036.pdf</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>历史985院校分类参考；非个人授位或就读当年建设身份的证明</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>未单独记录</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>scut</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>scut</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>华南理工大学</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G15"/>
+  <autoFilter ref="A1:G16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
@@ -3716,6 +4133,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>